<commit_message>
feat: add shinigami card image previews
</commit_message>
<xml_diff>
--- a/submissions/shinigami/config/shinigami_story_config.xlsx
+++ b/submissions/shinigami/config/shinigami_story_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhenxing\Documents\Codex\2026-05-22\codex-desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E944ED-E536-4432-8693-D74A60413D7B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2316242-2F20-4E65-A71D-76A110D8845B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="248">
   <si>
     <t>id</t>
   </si>
@@ -751,6 +751,109 @@
   </si>
   <si>
     <t>QI+0 SP+0 FN+0 RB-4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_2</t>
+  </si>
+  <si>
+    <t>card_2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_7</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_9</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_10</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_11</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_12</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_13</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_19</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_20</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_21</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_22</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_18</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_23</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_24</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_25</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_26</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_27</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_28</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>图片名</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1154,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -1168,7 +1271,7 @@
     <col min="11" max="11" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,8 +1305,11 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L1" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1233,8 +1339,11 @@
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-    </row>
-    <row r="3" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L2" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1264,8 +1373,11 @@
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
-    </row>
-    <row r="4" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L3" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1295,8 +1407,11 @@
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L4" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1328,8 +1443,11 @@
       <c r="K5" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L5" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1359,8 +1477,11 @@
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L6" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1390,8 +1511,11 @@
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L7" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1421,8 +1545,11 @@
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L8" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1452,8 +1579,11 @@
       </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L9" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1483,8 +1613,11 @@
       </c>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L10" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1518,8 +1651,11 @@
       <c r="K11" s="4" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L11" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1553,8 +1689,11 @@
       <c r="K12" s="4" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L12" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1584,8 +1723,11 @@
       </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L13" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1615,8 +1757,11 @@
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L14" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1650,8 +1795,11 @@
       <c r="K15" s="4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L15" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1685,8 +1833,11 @@
       <c r="K16" s="4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L16" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1716,8 +1867,11 @@
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L17" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1747,8 +1901,11 @@
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L18" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1782,8 +1939,11 @@
       <c r="K19" s="4" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L19" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1817,8 +1977,11 @@
       <c r="K20" s="4" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L20" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1850,8 +2013,11 @@
       <c r="K21" s="4" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L21" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1881,8 +2047,11 @@
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
-    </row>
-    <row r="23" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L22" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1916,8 +2085,11 @@
       <c r="K23" s="4" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L23" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1951,8 +2123,11 @@
       <c r="K24" s="4" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L24" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1982,8 +2157,11 @@
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
-    </row>
-    <row r="26" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L25" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -2013,8 +2191,11 @@
       </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
-    </row>
-    <row r="27" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L26" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -2048,8 +2229,11 @@
       <c r="K27" s="4" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L27" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -2083,8 +2267,11 @@
       <c r="K28" s="4" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L28" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -2114,8 +2301,11 @@
       </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
-    </row>
-    <row r="30" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L29" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2145,8 +2335,11 @@
       </c>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
-    </row>
-    <row r="31" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L30" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2180,8 +2373,11 @@
       <c r="K31" s="4" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L31" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2215,8 +2411,11 @@
       <c r="K32" s="4" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L32" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2246,10 +2445,14 @@
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
+      <c r="L33" s="2" t="s">
+        <v>224</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>